<commit_message>
agregado de notas de febrero
</commit_message>
<xml_diff>
--- a/inasistencias-4b-elecYsiscom-tp/alumnos-4b-ElecYsisCom-tp.xlsx
+++ b/inasistencias-4b-elecYsiscom-tp/alumnos-4b-ElecYsisCom-tp.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="657" uniqueCount="164">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="659" uniqueCount="166">
   <si>
     <t xml:space="preserve">nro</t>
   </si>
@@ -319,6 +319,9 @@
     <t xml:space="preserve">49837749@gmail.com</t>
   </si>
   <si>
+    <t xml:space="preserve">febrero</t>
+  </si>
+  <si>
     <t xml:space="preserve">1-fuentes</t>
   </si>
   <si>
@@ -413,6 +416,9 @@
   </si>
   <si>
     <t xml:space="preserve">separar los bornes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aprobado</t>
   </si>
   <si>
     <t xml:space="preserve">aporte de tevez</t>
@@ -550,12 +556,24 @@
       <family val="0"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor rgb="FFFFFF00"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00A933"/>
+        <bgColor rgb="FF008080"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -592,7 +610,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="11">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -613,11 +631,27 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -630,54 +664,7 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="13">
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF000000"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFCC0000"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFFFFF"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFCCFFCC"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF006600"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="7">
     <dxf>
       <font>
         <name val="Calibri"/>
@@ -744,7 +731,6 @@
           <bgColor rgb="FFCCFFCC"/>
         </patternFill>
       </fill>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </dxf>
     <dxf>
       <font>
@@ -759,7 +745,6 @@
           <bgColor rgb="FFFFCCCC"/>
         </patternFill>
       </fill>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </dxf>
     <dxf>
       <font>
@@ -775,7 +760,6 @@
           <bgColor rgb="FFCC0000"/>
         </patternFill>
       </fill>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </dxf>
   </dxfs>
   <colors>
@@ -829,7 +813,7 @@
       <rgbColor rgb="FF666699"/>
       <rgbColor rgb="FF969696"/>
       <rgbColor rgb="FF003366"/>
-      <rgbColor rgb="FF339966"/>
+      <rgbColor rgb="FF00A933"/>
       <rgbColor rgb="FF003300"/>
       <rgbColor rgb="FF333300"/>
       <rgbColor rgb="FF993300"/>
@@ -2639,7 +2623,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:AL19"/>
+  <dimension ref="A1:AN19"/>
   <sheetFormatPr defaultColWidth="9.5625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="4.32"/>
@@ -2667,10 +2651,10 @@
     <col collapsed="false" customWidth="false" hidden="true" outlineLevel="0" max="28" min="28" style="1" width="9.55"/>
     <col collapsed="false" customWidth="false" hidden="true" outlineLevel="0" max="29" min="29" style="1" width="9.56"/>
     <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="30" min="30" style="1" width="65.64"/>
-    <col collapsed="false" customWidth="false" hidden="true" outlineLevel="0" max="33" min="31" style="1" width="9.56"/>
-    <col collapsed="false" customWidth="false" hidden="true" outlineLevel="0" max="34" min="34" style="0" width="9.56"/>
+    <col collapsed="false" customWidth="false" hidden="true" outlineLevel="0" max="34" min="31" style="1" width="9.56"/>
     <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="35" min="35" style="1" width="20.92"/>
-    <col collapsed="false" customWidth="false" hidden="true" outlineLevel="0" max="37" min="36" style="0" width="9.56"/>
+    <col collapsed="false" customWidth="false" hidden="true" outlineLevel="0" max="37" min="36" style="1" width="9.56"/>
+    <col collapsed="false" customWidth="false" hidden="true" outlineLevel="0" max="38" min="38" style="0" width="9.56"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2681,6 +2665,9 @@
         <v>45835</v>
       </c>
       <c r="V1" s="3"/>
+      <c r="AM1" s="4" t="s">
+        <v>98</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
@@ -2693,37 +2680,37 @@
         <v>4</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="K2" s="1" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="L2" s="1" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="M2" s="1" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="N2" s="1" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="O2" s="1" t="s">
         <v>5</v>
@@ -2741,10 +2728,10 @@
         <v>5</v>
       </c>
       <c r="T2" s="1" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="U2" s="1" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="V2" s="3" t="n">
         <v>45898</v>
@@ -2788,11 +2775,14 @@
       <c r="AK2" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="AL2" s="4" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="AL2" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="AM2" s="5" t="n">
+        <v>46080</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="n">
         <v>1</v>
       </c>
@@ -2821,7 +2811,7 @@
         <f aca="false">G3+H3/2</f>
         <v>8</v>
       </c>
-      <c r="J3" s="5" t="n">
+      <c r="J3" s="6" t="n">
         <f aca="false">ROUND(AVERAGE(D3:F3,I3),0)</f>
         <v>5</v>
       </c>
@@ -2833,7 +2823,7 @@
         <v>7</v>
       </c>
       <c r="M3" s="1" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="N3" s="1" t="n">
         <v>7</v>
@@ -2848,7 +2838,7 @@
         <v>15</v>
       </c>
       <c r="S3" s="1" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="T3" s="1" t="n">
         <v>9</v>
@@ -2906,7 +2896,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="n">
         <v>2</v>
       </c>
@@ -2935,7 +2925,7 @@
         <f aca="false">G4+H4/2</f>
         <v>8</v>
       </c>
-      <c r="J4" s="5" t="n">
+      <c r="J4" s="6" t="n">
         <f aca="false">ROUND(AVERAGE(D4:F4,I4),0)</f>
         <v>6</v>
       </c>
@@ -2947,7 +2937,7 @@
         <v>8</v>
       </c>
       <c r="M4" s="1" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="N4" s="1" t="n">
         <v>7</v>
@@ -2962,7 +2952,7 @@
         <v>15</v>
       </c>
       <c r="S4" s="1" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="T4" s="1" t="n">
         <v>10</v>
@@ -3009,7 +2999,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="n">
         <v>3</v>
       </c>
@@ -3038,7 +3028,7 @@
         <f aca="false">G5+H5/2</f>
         <v>9</v>
       </c>
-      <c r="J5" s="5" t="n">
+      <c r="J5" s="6" t="n">
         <f aca="false">ROUND(AVERAGE(D5:F5,I5),0)</f>
         <v>8</v>
       </c>
@@ -3050,13 +3040,13 @@
         <v>7</v>
       </c>
       <c r="M5" s="1" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="N5" s="1" t="n">
         <v>8</v>
       </c>
       <c r="O5" s="1" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="P5" s="1" t="n">
         <v>6</v>
@@ -3124,7 +3114,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="n">
         <v>4</v>
       </c>
@@ -3153,7 +3143,7 @@
         <f aca="false">G6+H6/2</f>
         <v>8</v>
       </c>
-      <c r="J6" s="5" t="n">
+      <c r="J6" s="6" t="n">
         <f aca="false">ROUND(AVERAGE(D6:F6,I6),0)</f>
         <v>6</v>
       </c>
@@ -3165,7 +3155,7 @@
         <v>7</v>
       </c>
       <c r="M6" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="N6" s="1" t="n">
         <v>8</v>
@@ -3221,7 +3211,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="n">
         <v>5</v>
       </c>
@@ -3250,7 +3240,7 @@
         <f aca="false">G7+H7/2</f>
         <v>8</v>
       </c>
-      <c r="J7" s="5" t="n">
+      <c r="J7" s="6" t="n">
         <f aca="false">ROUND(AVERAGE(D7:F7,I7),0)</f>
         <v>8</v>
       </c>
@@ -3262,7 +3252,7 @@
         <v>7</v>
       </c>
       <c r="M7" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="N7" s="1" t="n">
         <v>8</v>
@@ -3296,7 +3286,7 @@
         <v>7</v>
       </c>
       <c r="AD7" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AE7" s="1" t="s">
         <v>15</v>
@@ -3321,7 +3311,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="n">
         <v>6</v>
       </c>
@@ -3350,7 +3340,7 @@
         <f aca="false">G8+H8/2</f>
         <v>8</v>
       </c>
-      <c r="J8" s="5" t="n">
+      <c r="J8" s="6" t="n">
         <f aca="false">ROUND(AVERAGE(D8:F8,I8),0)</f>
         <v>5</v>
       </c>
@@ -3362,7 +3352,7 @@
         <v>8</v>
       </c>
       <c r="M8" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="N8" s="1" t="n">
         <v>7</v>
@@ -3377,7 +3367,7 @@
         <v>15</v>
       </c>
       <c r="S8" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="T8" s="1" t="n">
         <v>9</v>
@@ -3427,7 +3417,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="n">
         <v>7</v>
       </c>
@@ -3456,7 +3446,7 @@
         <f aca="false">G9+H9/2</f>
         <v>8</v>
       </c>
-      <c r="J9" s="5" t="n">
+      <c r="J9" s="6" t="n">
         <f aca="false">ROUND(AVERAGE(D9:F9,I9),0)</f>
         <v>6</v>
       </c>
@@ -3468,13 +3458,13 @@
         <v>7</v>
       </c>
       <c r="M9" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="N9" s="1" t="n">
         <v>7</v>
       </c>
       <c r="O9" s="1" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="P9" s="1" t="n">
         <v>6</v>
@@ -3486,7 +3476,7 @@
         <v>15</v>
       </c>
       <c r="S9" s="1" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="T9" s="1" t="n">
         <v>9</v>
@@ -3545,7 +3535,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="n">
         <v>8</v>
       </c>
@@ -3574,7 +3564,7 @@
         <f aca="false">G10+H10/2</f>
         <v>1</v>
       </c>
-      <c r="J10" s="5" t="n">
+      <c r="J10" s="6" t="n">
         <f aca="false">ROUND(AVERAGE(D10:F10,I10),0)</f>
         <v>3</v>
       </c>
@@ -3586,7 +3576,7 @@
         <v>7</v>
       </c>
       <c r="M10" s="1" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="N10" s="1" t="n">
         <v>8</v>
@@ -3601,7 +3591,7 @@
         <v>27</v>
       </c>
       <c r="S10" s="1" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="T10" s="1" t="n">
         <v>9</v>
@@ -3654,7 +3644,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="n">
         <v>9</v>
       </c>
@@ -3683,7 +3673,7 @@
         <f aca="false">G11+H11/2</f>
         <v>8</v>
       </c>
-      <c r="J11" s="5" t="n">
+      <c r="J11" s="6" t="n">
         <f aca="false">ROUND(AVERAGE(D11:F11,I11),0)</f>
         <v>8</v>
       </c>
@@ -3754,7 +3744,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="n">
         <v>10</v>
       </c>
@@ -3783,7 +3773,7 @@
         <f aca="false">G12+H12/2</f>
         <v>8</v>
       </c>
-      <c r="J12" s="5" t="n">
+      <c r="J12" s="6" t="n">
         <f aca="false">ROUND(AVERAGE(D12:F12,I12),0)</f>
         <v>6</v>
       </c>
@@ -3795,13 +3785,13 @@
         <v>7</v>
       </c>
       <c r="M12" s="1" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="N12" s="1" t="n">
         <v>7</v>
       </c>
       <c r="O12" s="1" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="P12" s="1" t="n">
         <v>6</v>
@@ -3813,7 +3803,7 @@
         <v>15</v>
       </c>
       <c r="S12" s="1" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="T12" s="1" t="n">
         <v>9</v>
@@ -3863,7 +3853,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="n">
         <v>11</v>
       </c>
@@ -3892,7 +3882,7 @@
         <f aca="false">G13+H13/2</f>
         <v>8</v>
       </c>
-      <c r="J13" s="5" t="n">
+      <c r="J13" s="6" t="n">
         <f aca="false">ROUND(AVERAGE(D13:F13,I13),0)</f>
         <v>5</v>
       </c>
@@ -3957,7 +3947,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="n">
         <v>12</v>
       </c>
@@ -3986,7 +3976,7 @@
         <f aca="false">G14+H14/2</f>
         <v>8</v>
       </c>
-      <c r="J14" s="5" t="n">
+      <c r="J14" s="6" t="n">
         <f aca="false">ROUND(AVERAGE(D14:F14,I14),0)</f>
         <v>7</v>
       </c>
@@ -3998,7 +3988,7 @@
         <v>7</v>
       </c>
       <c r="M14" s="1" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="N14" s="1" t="n">
         <v>7</v>
@@ -4054,7 +4044,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="n">
         <v>13</v>
       </c>
@@ -4083,7 +4073,7 @@
         <f aca="false">G15+H15/2</f>
         <v>9</v>
       </c>
-      <c r="J15" s="5" t="n">
+      <c r="J15" s="6" t="n">
         <f aca="false">ROUND(AVERAGE(D15:F15,I15),0)</f>
         <v>6</v>
       </c>
@@ -4129,7 +4119,7 @@
         <v>8</v>
       </c>
       <c r="AD15" s="1" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="AE15" s="1" t="s">
         <v>15</v>
@@ -4154,116 +4144,122 @@
         <v>8</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="1" t="n">
+    <row r="16" s="7" customFormat="true" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="7" t="n">
         <v>14</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="B16" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="C16" s="1" t="s">
+      <c r="C16" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="D16" s="1" t="n">
+      <c r="D16" s="9" t="n">
+        <v>7</v>
+      </c>
+      <c r="E16" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="F16" s="9" t="n">
+        <v>7</v>
+      </c>
+      <c r="G16" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="E16" s="1" t="n">
-        <v>6</v>
-      </c>
-      <c r="F16" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="G16" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="H16" s="1" t="n">
+      <c r="H16" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="I16" s="1" t="n">
+      <c r="I16" s="7" t="n">
         <f aca="false">G16+H16/2</f>
         <v>1</v>
       </c>
-      <c r="J16" s="5" t="n">
+      <c r="J16" s="10" t="n">
         <f aca="false">ROUND(AVERAGE(D16:F16,I16),0)</f>
-        <v>2</v>
-      </c>
-      <c r="K16" s="1" t="str">
+        <v>5</v>
+      </c>
+      <c r="K16" s="7" t="str">
         <f aca="false">IF(J16&lt;7,"TEP","TEA")</f>
         <v>TEP</v>
       </c>
-      <c r="L16" s="1" t="n">
-        <v>7</v>
-      </c>
-      <c r="N16" s="1" t="n">
-        <v>8</v>
-      </c>
-      <c r="P16" s="1" t="n">
-        <v>7</v>
-      </c>
-      <c r="Q16" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="R16" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="S16" s="1" t="s">
-        <v>129</v>
-      </c>
-      <c r="T16" s="1" t="n">
-        <v>7</v>
-      </c>
-      <c r="U16" s="1" t="n">
+      <c r="L16" s="7" t="n">
+        <v>7</v>
+      </c>
+      <c r="N16" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="P16" s="7" t="n">
+        <v>7</v>
+      </c>
+      <c r="Q16" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="R16" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="S16" s="7" t="s">
+        <v>130</v>
+      </c>
+      <c r="T16" s="7" t="n">
+        <v>7</v>
+      </c>
+      <c r="U16" s="10" t="n">
         <f aca="false">ROUND(AVERAGE(T16,R16,P16,N16,L16),0)</f>
         <v>7</v>
       </c>
-      <c r="W16" s="1" t="n">
-        <v>6</v>
-      </c>
-      <c r="X16" s="1" t="s">
+      <c r="W16" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="X16" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="Y16" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="Z16" s="1" t="n">
+      <c r="Y16" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="Z16" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="AA16" s="1" t="s">
+      <c r="AA16" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="AB16" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="AC16" s="1" t="n">
+      <c r="AB16" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="AC16" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="AD16" s="1" t="s">
+      <c r="AD16" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="AE16" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="AF16" s="1" t="n">
+      <c r="AE16" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="AF16" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="AG16" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="AH16" s="1" t="n">
+      <c r="AG16" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="AH16" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="AI16" s="2" t="s">
+      <c r="AI16" s="8" t="s">
         <v>45</v>
       </c>
-      <c r="AJ16" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="AK16" s="1" t="n">
+      <c r="AJ16" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="AK16" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="AL16" s="6" t="n">
+      <c r="AL16" s="10" t="n">
         <f aca="false">ROUND(AVERAGE(AK16,AH16,AF16,AC16,Z16,W16,C16),0)</f>
         <v>3</v>
+      </c>
+      <c r="AM16" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="AN16" s="7" t="s">
+        <v>131</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4295,7 +4291,7 @@
         <f aca="false">G17+H17/2</f>
         <v>1</v>
       </c>
-      <c r="J17" s="5" t="n">
+      <c r="J17" s="6" t="n">
         <f aca="false">ROUND(AVERAGE(D17:F17,I17),0)</f>
         <v>2</v>
       </c>
@@ -4319,7 +4315,7 @@
         <v>27</v>
       </c>
       <c r="S17" s="1" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="T17" s="1" t="n">
         <v>1</v>
@@ -4366,7 +4362,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" ht="15.65" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="n">
         <v>16</v>
       </c>
@@ -4395,7 +4391,7 @@
         <f aca="false">G18+H18/2</f>
         <v>8</v>
       </c>
-      <c r="J18" s="5" t="n">
+      <c r="J18" s="6" t="n">
         <f aca="false">ROUND(AVERAGE(D18:F18,I18),0)</f>
         <v>6</v>
       </c>
@@ -4492,36 +4488,36 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="J3:J18">
-    <cfRule type="cellIs" priority="2" operator="lessThan" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="6">
+    <cfRule type="cellIs" priority="2" operator="lessThan" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
       <formula>7</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K3:K18">
-    <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="6">
+    <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
       <formula>"TEP"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="U3:U18">
-    <cfRule type="cellIs" priority="4" operator="greaterThan" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
+    <cfRule type="cellIs" priority="4" operator="greaterThan" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
       <formula>6</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="5" operator="notBetween" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
+    <cfRule type="cellIs" priority="5" operator="notBetween" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="2">
       <formula>4</formula>
       <formula>6</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="6" operator="lessThan" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="9">
+    <cfRule type="cellIs" priority="6" operator="lessThan" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="3">
       <formula>4</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AL3:AL18">
-    <cfRule type="cellIs" priority="7" operator="greaterThan" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="10">
+    <cfRule type="cellIs" priority="7" operator="greaterThan" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="4">
       <formula>6</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="8" operator="between" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="11">
+    <cfRule type="cellIs" priority="8" operator="between" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="5">
       <formula>4</formula>
       <formula>6</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="9" operator="lessThan" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="12">
+    <cfRule type="cellIs" priority="9" operator="lessThan" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="6">
       <formula>4</formula>
     </cfRule>
   </conditionalFormatting>
@@ -4553,22 +4549,22 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4596,10 +4592,10 @@
         <v>57</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="F3" s="1" t="n">
         <v>8</v>
@@ -4619,10 +4615,10 @@
         <v>12</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="F4" s="1" t="n">
         <v>5</v>
@@ -4642,10 +4638,10 @@
         <v>25</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="F5" s="1" t="n">
         <v>7</v>
@@ -4665,10 +4661,10 @@
         <v>29</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="F6" s="1" t="n">
         <v>7</v>
@@ -4688,10 +4684,10 @@
         <v>62</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="F7" s="1" t="n">
         <v>3</v>
@@ -4711,10 +4707,10 @@
         <v>77</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="F8" s="1" t="n">
         <v>9</v>
@@ -4736,10 +4732,10 @@
         <v>77</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="F9" s="1" t="n">
         <v>1</v>
@@ -4756,10 +4752,10 @@
         <v>36</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="F10" s="1" t="n">
         <v>2</v>
@@ -4779,10 +4775,10 @@
         <v>68</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="F11" s="1" t="n">
         <v>7</v>
@@ -4802,10 +4798,10 @@
         <v>87</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="F12" s="1" t="n">
         <v>7</v>
@@ -4827,10 +4823,10 @@
         <v>87</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="F13" s="1" t="n">
         <v>5</v>
@@ -4847,10 +4843,10 @@
         <v>73</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="F14" s="1" t="n">
         <v>1</v>
@@ -4870,10 +4866,10 @@
         <v>92</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="F15" s="1" t="n">
         <v>2</v>
@@ -4893,10 +4889,10 @@
         <v>96</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="F16" s="1" t="n">
         <v>6</v>
@@ -4916,10 +4912,10 @@
         <v>42</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="F17" s="1" t="n">
         <v>1</v>
@@ -4953,10 +4949,10 @@
         <v>32</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="F19" s="1" t="n">
         <v>7</v>
@@ -5001,10 +4997,10 @@
         <v>45751</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>